<commit_message>
Edits to standardized variables after 2025 CI report
</commit_message>
<xml_diff>
--- a/Data/2011_F033_CO_RSIS/2011_F033_CO_RSIS_SoilChemistry.xlsx
+++ b/Data/2011_F033_CO_RSIS/2011_F033_CO_RSIS_SoilChemistry.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI project\cottondata\Data\2011_F033_CO_RSIS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4971CB24-74B4-4E03-85E4-FAF488254EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CBBFE07-8B67-493C-A41A-42CF0C231DF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16260" yWindow="-27495" windowWidth="17910" windowHeight="26685" xr2:uid="{EDD8493E-22F9-4363-B206-02BA4DA4CD3D}"/>
+    <workbookView xWindow="-1815" yWindow="-26850" windowWidth="16230" windowHeight="26310" xr2:uid="{EDD8493E-22F9-4363-B206-02BA4DA4CD3D}"/>
   </bookViews>
   <sheets>
     <sheet name="SoilChemDF" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="991" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="992" uniqueCount="321">
   <si>
     <t>FB</t>
   </si>
@@ -1006,6 +1006,9 @@
   </si>
   <si>
     <t>p16-6</t>
+  </si>
+  <si>
+    <t>Depth2</t>
   </si>
 </sst>
 </file>
@@ -2801,13 +2804,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4750B6AC-9758-417A-92D8-714809E6735E}">
-  <dimension ref="A1:F145"/>
+  <dimension ref="A1:G145"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>266</v>
       </c>
@@ -2826,8 +2829,11 @@
       <c r="F1" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2011</v>
       </c>
@@ -2846,8 +2852,12 @@
       <c r="F2" s="62">
         <v>0.54</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2">
+        <f>E2-15</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2011</v>
       </c>
@@ -2866,8 +2876,12 @@
       <c r="F3" s="62">
         <v>1.65</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3">
+        <f t="shared" ref="G3:G66" si="0">E3-15</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2011</v>
       </c>
@@ -2886,8 +2900,12 @@
       <c r="F4" s="62">
         <v>2.5499999999999998</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2011</v>
       </c>
@@ -2906,8 +2924,12 @@
       <c r="F5" s="62">
         <v>1.44</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2011</v>
       </c>
@@ -2926,8 +2948,12 @@
       <c r="F6" s="62">
         <v>3.34</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2011</v>
       </c>
@@ -2946,8 +2972,12 @@
       <c r="F7" s="62">
         <v>3.18</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2011</v>
       </c>
@@ -2966,8 +2996,12 @@
       <c r="F8" s="62">
         <v>6.38</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2011</v>
       </c>
@@ -2986,8 +3020,12 @@
       <c r="F9" s="62">
         <v>2.38</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2011</v>
       </c>
@@ -3006,8 +3044,12 @@
       <c r="F10" s="62">
         <v>9.66</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2011</v>
       </c>
@@ -3026,8 +3068,12 @@
       <c r="F11" s="62">
         <v>5.28</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2011</v>
       </c>
@@ -3046,8 +3092,12 @@
       <c r="F12" s="62">
         <v>9.0500000000000007</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2011</v>
       </c>
@@ -3066,8 +3116,12 @@
       <c r="F13" s="62">
         <v>10.99</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2011</v>
       </c>
@@ -3086,8 +3140,12 @@
       <c r="F14" s="62">
         <v>9.52</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2011</v>
       </c>
@@ -3106,8 +3164,12 @@
       <c r="F15" s="62">
         <v>7.08</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2011</v>
       </c>
@@ -3126,8 +3188,12 @@
       <c r="F16" s="62">
         <v>7.96</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2011</v>
       </c>
@@ -3146,8 +3212,12 @@
       <c r="F17" s="62">
         <v>9.09</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2011</v>
       </c>
@@ -3166,8 +3236,12 @@
       <c r="F18" s="62">
         <v>4.5</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2011</v>
       </c>
@@ -3186,8 +3260,12 @@
       <c r="F19" s="62">
         <v>4.0599999999999996</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2011</v>
       </c>
@@ -3206,8 +3284,12 @@
       <c r="F20" s="62">
         <v>2.06</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2011</v>
       </c>
@@ -3226,8 +3308,12 @@
       <c r="F21" s="62">
         <v>4.8899999999999997</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G21">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2011</v>
       </c>
@@ -3246,8 +3332,12 @@
       <c r="F22" s="62">
         <v>2.82</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G22">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2011</v>
       </c>
@@ -3266,8 +3356,12 @@
       <c r="F23" s="62">
         <v>0.78</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G23">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2011</v>
       </c>
@@ -3286,8 +3380,12 @@
       <c r="F24" s="62">
         <v>1.25</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G24">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2011</v>
       </c>
@@ -3306,8 +3404,12 @@
       <c r="F25" s="62">
         <v>2.21</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G25">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2011</v>
       </c>
@@ -3326,8 +3428,12 @@
       <c r="F26" s="62">
         <v>7.46</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G26">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2011</v>
       </c>
@@ -3346,8 +3452,12 @@
       <c r="F27" s="62">
         <v>4.2</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G27">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2011</v>
       </c>
@@ -3366,8 +3476,12 @@
       <c r="F28" s="62">
         <v>7.02</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G28">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2011</v>
       </c>
@@ -3386,8 +3500,12 @@
       <c r="F29" s="62">
         <v>8.91</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G29">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2011</v>
       </c>
@@ -3406,8 +3524,12 @@
       <c r="F30" s="62">
         <v>9.33</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G30">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2011</v>
       </c>
@@ -3426,8 +3548,12 @@
       <c r="F31" s="62">
         <v>15.89</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G31">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2011</v>
       </c>
@@ -3446,8 +3572,12 @@
       <c r="F32" s="62">
         <v>14.96</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G32">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2011</v>
       </c>
@@ -3466,8 +3596,12 @@
       <c r="F33" s="62">
         <v>29.68</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G33">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2011</v>
       </c>
@@ -3486,8 +3620,12 @@
       <c r="F34" s="62">
         <v>10.66</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G34">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2011</v>
       </c>
@@ -3506,8 +3644,12 @@
       <c r="F35" s="62">
         <v>4.62</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G35">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>2011</v>
       </c>
@@ -3526,8 +3668,12 @@
       <c r="F36" s="62">
         <v>2.33</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G36">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>2011</v>
       </c>
@@ -3546,8 +3692,12 @@
       <c r="F37" s="62">
         <v>2.82</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G37">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>2011</v>
       </c>
@@ -3566,8 +3716,12 @@
       <c r="F38" s="62">
         <v>2.84</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G38">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2011</v>
       </c>
@@ -3586,8 +3740,12 @@
       <c r="F39" s="62">
         <v>3.14</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G39">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>2011</v>
       </c>
@@ -3606,8 +3764,12 @@
       <c r="F40" s="62">
         <v>4.4800000000000004</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G40">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2011</v>
       </c>
@@ -3626,8 +3788,12 @@
       <c r="F41" s="62">
         <v>2.5299999999999998</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G41">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>2011</v>
       </c>
@@ -3646,8 +3812,12 @@
       <c r="F42" s="62">
         <v>7.8</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G42">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>2011</v>
       </c>
@@ -3666,8 +3836,12 @@
       <c r="F43" s="62">
         <v>3.09</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G43">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>2011</v>
       </c>
@@ -3686,8 +3860,12 @@
       <c r="F44" s="62">
         <v>10.3</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G44">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>2011</v>
       </c>
@@ -3706,8 +3884,12 @@
       <c r="F45" s="62">
         <v>8.2200000000000006</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G45">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>2011</v>
       </c>
@@ -3726,8 +3908,12 @@
       <c r="F46" s="62">
         <v>3.38</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G46">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>2011</v>
       </c>
@@ -3746,8 +3932,12 @@
       <c r="F47" s="62">
         <v>11.44</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G47">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2011</v>
       </c>
@@ -3766,8 +3956,12 @@
       <c r="F48" s="62">
         <v>12.99</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G48">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>2011</v>
       </c>
@@ -3786,8 +3980,12 @@
       <c r="F49" s="62">
         <v>17.64</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G49">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>2011</v>
       </c>
@@ -3806,8 +4004,12 @@
       <c r="F50" s="62">
         <v>15.9</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G50">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>2011</v>
       </c>
@@ -3826,8 +4028,12 @@
       <c r="F51" s="62">
         <v>16.559999999999999</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G51">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>2011</v>
       </c>
@@ -3846,8 +4052,12 @@
       <c r="F52" s="62">
         <v>11.08</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G52">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>2011</v>
       </c>
@@ -3866,8 +4076,12 @@
       <c r="F53" s="62">
         <v>14.43</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G53">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>2011</v>
       </c>
@@ -3886,8 +4100,12 @@
       <c r="F54" s="62">
         <v>8.85</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G54">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>2011</v>
       </c>
@@ -3906,8 +4124,12 @@
       <c r="F55" s="62">
         <v>2.4700000000000002</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G55">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>2011</v>
       </c>
@@ -3926,8 +4148,12 @@
       <c r="F56" s="62">
         <v>12.08</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G56">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>2011</v>
       </c>
@@ -3946,8 +4172,12 @@
       <c r="F57" s="62">
         <v>9.43</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G57">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>2011</v>
       </c>
@@ -3966,8 +4196,12 @@
       <c r="F58" s="62">
         <v>1.95</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G58">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>2011</v>
       </c>
@@ -3986,8 +4220,12 @@
       <c r="F59" s="62">
         <v>13.59</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G59">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>2011</v>
       </c>
@@ -4006,8 +4244,12 @@
       <c r="F60" s="62">
         <v>11.23</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G60">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>2011</v>
       </c>
@@ -4026,8 +4268,12 @@
       <c r="F61" s="62">
         <v>10.74</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G61">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>2011</v>
       </c>
@@ -4046,8 +4292,12 @@
       <c r="F62" s="62">
         <v>12.77</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G62">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>2011</v>
       </c>
@@ -4066,8 +4316,12 @@
       <c r="F63" s="62">
         <v>7.2</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G63">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>2011</v>
       </c>
@@ -4086,8 +4340,12 @@
       <c r="F64" s="62">
         <v>2.4</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G64">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>2011</v>
       </c>
@@ -4106,8 +4364,12 @@
       <c r="F65" s="62">
         <v>29.19</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G65">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>2011</v>
       </c>
@@ -4126,8 +4388,12 @@
       <c r="F66" s="62">
         <v>24.34</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G66">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>2011</v>
       </c>
@@ -4146,8 +4412,12 @@
       <c r="F67" s="62">
         <v>15.7</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G67">
+        <f t="shared" ref="G67:G130" si="1">E67-15</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>2011</v>
       </c>
@@ -4166,8 +4436,12 @@
       <c r="F68" s="62">
         <v>13.88</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G68">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>2011</v>
       </c>
@@ -4186,8 +4460,12 @@
       <c r="F69" s="62">
         <v>10.35</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G69">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>2011</v>
       </c>
@@ -4206,8 +4484,12 @@
       <c r="F70" s="62">
         <v>6.84</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G70">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>2011</v>
       </c>
@@ -4226,8 +4508,12 @@
       <c r="F71" s="62">
         <v>18.760000000000002</v>
       </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G71">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>2011</v>
       </c>
@@ -4246,8 +4532,12 @@
       <c r="F72" s="62">
         <v>7.39</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G72">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>2011</v>
       </c>
@@ -4266,8 +4556,12 @@
       <c r="F73" s="62">
         <v>2.36</v>
       </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G73">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>2011</v>
       </c>
@@ -4286,8 +4580,12 @@
       <c r="F74" s="62">
         <v>9.4700000000000006</v>
       </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G74">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>2011</v>
       </c>
@@ -4306,8 +4604,12 @@
       <c r="F75" s="62">
         <v>7.44</v>
       </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G75">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>2011</v>
       </c>
@@ -4326,8 +4628,12 @@
       <c r="F76" s="62">
         <v>5.64</v>
       </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G76">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>2011</v>
       </c>
@@ -4346,8 +4652,12 @@
       <c r="F77" s="62">
         <v>20.48</v>
       </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G77">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>2011</v>
       </c>
@@ -4366,8 +4676,12 @@
       <c r="F78" s="62">
         <v>5.17</v>
       </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G78">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>2011</v>
       </c>
@@ -4386,8 +4700,12 @@
       <c r="F79" s="62">
         <v>3.45</v>
       </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G79">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>2011</v>
       </c>
@@ -4406,8 +4724,12 @@
       <c r="F80" s="62">
         <v>9.82</v>
       </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G80">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>2011</v>
       </c>
@@ -4426,8 +4748,12 @@
       <c r="F81" s="62">
         <v>10.46</v>
       </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G81">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>2011</v>
       </c>
@@ -4446,8 +4772,12 @@
       <c r="F82" s="62">
         <v>13.55</v>
       </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G82">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>2011</v>
       </c>
@@ -4466,8 +4796,12 @@
       <c r="F83" s="62">
         <v>21.27</v>
       </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G83">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>2011</v>
       </c>
@@ -4486,8 +4820,12 @@
       <c r="F84" s="62">
         <v>18.54</v>
       </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G84">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>2011</v>
       </c>
@@ -4506,8 +4844,12 @@
       <c r="F85" s="62">
         <v>19.45</v>
       </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G85">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>2011</v>
       </c>
@@ -4526,8 +4868,12 @@
       <c r="F86" s="62">
         <v>19.84</v>
       </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G86">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>2011</v>
       </c>
@@ -4546,8 +4892,12 @@
       <c r="F87" s="62">
         <v>18.95</v>
       </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G87">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>2011</v>
       </c>
@@ -4566,8 +4916,12 @@
       <c r="F88" s="62">
         <v>15.55</v>
       </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G88">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>2011</v>
       </c>
@@ -4586,8 +4940,12 @@
       <c r="F89" s="62">
         <v>15.62</v>
       </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G89">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>2011</v>
       </c>
@@ -4606,8 +4964,12 @@
       <c r="F90" s="62">
         <v>10.49</v>
       </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G90">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>2011</v>
       </c>
@@ -4626,8 +4988,12 @@
       <c r="F91" s="62">
         <v>10.5</v>
       </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G91">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>2011</v>
       </c>
@@ -4646,8 +5012,12 @@
       <c r="F92" s="62">
         <v>11.44</v>
       </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G92">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>2011</v>
       </c>
@@ -4666,8 +5036,12 @@
       <c r="F93" s="62">
         <v>15.62</v>
       </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G93">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>2011</v>
       </c>
@@ -4686,8 +5060,12 @@
       <c r="F94" s="62">
         <v>14.12</v>
       </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G94">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>2011</v>
       </c>
@@ -4706,8 +5084,12 @@
       <c r="F95" s="62">
         <v>17.920000000000002</v>
       </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G95">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>2011</v>
       </c>
@@ -4726,8 +5108,12 @@
       <c r="F96" s="62">
         <v>7.47</v>
       </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G96">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>2011</v>
       </c>
@@ -4746,8 +5132,12 @@
       <c r="F97" s="62">
         <v>2.61</v>
       </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G97">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>2011</v>
       </c>
@@ -4766,8 +5156,12 @@
       <c r="F98" s="62">
         <v>21.94</v>
       </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G98">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>2011</v>
       </c>
@@ -4786,8 +5180,12 @@
       <c r="F99" s="62">
         <v>9.7100000000000009</v>
       </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G99">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>2011</v>
       </c>
@@ -4806,8 +5204,12 @@
       <c r="F100" s="62">
         <v>3.65</v>
       </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G100">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>2011</v>
       </c>
@@ -4826,8 +5228,12 @@
       <c r="F101" s="62">
         <v>15.19</v>
       </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G101">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>2011</v>
       </c>
@@ -4846,8 +5252,12 @@
       <c r="F102" s="62">
         <v>10.27</v>
       </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G102">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>2011</v>
       </c>
@@ -4866,8 +5276,12 @@
       <c r="F103" s="62">
         <v>11.17</v>
       </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G103">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>2011</v>
       </c>
@@ -4886,8 +5300,12 @@
       <c r="F104" s="62">
         <v>33.729999999999997</v>
       </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G104">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>2011</v>
       </c>
@@ -4906,8 +5324,12 @@
       <c r="F105" s="62">
         <v>18.059999999999999</v>
       </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G105">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>2011</v>
       </c>
@@ -4926,8 +5348,12 @@
       <c r="F106" s="62">
         <v>10.52</v>
       </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G106">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>2011</v>
       </c>
@@ -4946,8 +5372,12 @@
       <c r="F107" s="62">
         <v>30.43</v>
       </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G107">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>2011</v>
       </c>
@@ -4966,8 +5396,12 @@
       <c r="F108" s="62">
         <v>8.61</v>
       </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G108">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>2011</v>
       </c>
@@ -4986,8 +5420,12 @@
       <c r="F109" s="62">
         <v>6.95</v>
       </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G109">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>2011</v>
       </c>
@@ -5006,8 +5444,12 @@
       <c r="F110" s="62">
         <v>39.85</v>
       </c>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G110">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>2011</v>
       </c>
@@ -5026,8 +5468,12 @@
       <c r="F111" s="62">
         <v>14.24</v>
       </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G111">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>2011</v>
       </c>
@@ -5046,8 +5492,12 @@
       <c r="F112" s="62">
         <v>5.4</v>
       </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G112">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>2011</v>
       </c>
@@ -5066,8 +5516,12 @@
       <c r="F113" s="62">
         <v>15.47</v>
       </c>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G113">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>2011</v>
       </c>
@@ -5086,8 +5540,12 @@
       <c r="F114" s="62">
         <v>8.36</v>
       </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G114">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>2011</v>
       </c>
@@ -5106,8 +5564,12 @@
       <c r="F115" s="62">
         <v>9.14</v>
       </c>
-    </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G115">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>2011</v>
       </c>
@@ -5126,8 +5588,12 @@
       <c r="F116" s="62">
         <v>11.18</v>
       </c>
-    </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G116">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>2011</v>
       </c>
@@ -5146,8 +5612,12 @@
       <c r="F117" s="62">
         <v>7.21</v>
       </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G117">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>2011</v>
       </c>
@@ -5166,8 +5636,12 @@
       <c r="F118" s="62">
         <v>2.41</v>
       </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G118">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>2011</v>
       </c>
@@ -5186,8 +5660,12 @@
       <c r="F119" s="62">
         <v>30.78</v>
       </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G119">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>2011</v>
       </c>
@@ -5206,8 +5684,12 @@
       <c r="F120" s="62">
         <v>6.57</v>
       </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G120">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>2011</v>
       </c>
@@ -5226,8 +5708,12 @@
       <c r="F121" s="62">
         <v>4.58</v>
       </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G121">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>2011</v>
       </c>
@@ -5246,8 +5732,12 @@
       <c r="F122" s="62">
         <v>14.06</v>
       </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G122">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>2011</v>
       </c>
@@ -5266,8 +5756,12 @@
       <c r="F123" s="62">
         <v>5.81</v>
       </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G123">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>2011</v>
       </c>
@@ -5286,8 +5780,12 @@
       <c r="F124" s="62">
         <v>2.61</v>
       </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G124">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>2011</v>
       </c>
@@ -5306,8 +5804,12 @@
       <c r="F125" s="62">
         <v>14.7</v>
       </c>
-    </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G125">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>2011</v>
       </c>
@@ -5326,8 +5828,12 @@
       <c r="F126" s="62">
         <v>5.1100000000000003</v>
       </c>
-    </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G126">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>2011</v>
       </c>
@@ -5346,8 +5852,12 @@
       <c r="F127" s="62">
         <v>4.9400000000000004</v>
       </c>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G127">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>2011</v>
       </c>
@@ -5366,8 +5876,12 @@
       <c r="F128" s="62">
         <v>9.68</v>
       </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G128">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>2011</v>
       </c>
@@ -5386,8 +5900,12 @@
       <c r="F129" s="62">
         <v>5.9</v>
       </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G129">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>2011</v>
       </c>
@@ -5406,8 +5924,12 @@
       <c r="F130" s="62">
         <v>2.11</v>
       </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G130">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>2011</v>
       </c>
@@ -5426,8 +5948,12 @@
       <c r="F131" s="62">
         <v>11.51</v>
       </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G131">
+        <f t="shared" ref="G131:G145" si="2">E131-15</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>2011</v>
       </c>
@@ -5446,8 +5972,12 @@
       <c r="F132" s="62">
         <v>9.25</v>
       </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G132">
+        <f t="shared" si="2"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>2011</v>
       </c>
@@ -5466,8 +5996,12 @@
       <c r="F133" s="62">
         <v>6.78</v>
       </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G133">
+        <f t="shared" si="2"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>2011</v>
       </c>
@@ -5486,8 +6020,12 @@
       <c r="F134" s="62">
         <v>10.37</v>
       </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G134">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>2011</v>
       </c>
@@ -5506,8 +6044,12 @@
       <c r="F135" s="62">
         <v>5.36</v>
       </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G135">
+        <f t="shared" si="2"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>2011</v>
       </c>
@@ -5526,8 +6068,12 @@
       <c r="F136" s="62">
         <v>8.99</v>
       </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G136">
+        <f t="shared" si="2"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>2011</v>
       </c>
@@ -5546,8 +6092,12 @@
       <c r="F137" s="62">
         <v>12.17</v>
       </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G137">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>2011</v>
       </c>
@@ -5566,8 +6116,12 @@
       <c r="F138" s="62">
         <v>9.2799999999999994</v>
       </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G138">
+        <f t="shared" si="2"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>2011</v>
       </c>
@@ -5586,8 +6140,12 @@
       <c r="F139" s="62">
         <v>3.23</v>
       </c>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G139">
+        <f t="shared" si="2"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>2011</v>
       </c>
@@ -5606,8 +6164,12 @@
       <c r="F140" s="62">
         <v>11.11</v>
       </c>
-    </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G140">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>2011</v>
       </c>
@@ -5626,8 +6188,12 @@
       <c r="F141" s="62">
         <v>19.2</v>
       </c>
-    </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G141">
+        <f t="shared" si="2"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>2011</v>
       </c>
@@ -5646,8 +6212,12 @@
       <c r="F142" s="62">
         <v>2.34</v>
       </c>
-    </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G142">
+        <f t="shared" si="2"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>2011</v>
       </c>
@@ -5666,8 +6236,12 @@
       <c r="F143" s="62">
         <v>11.47</v>
       </c>
-    </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G143">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>2011</v>
       </c>
@@ -5686,8 +6260,12 @@
       <c r="F144" s="62">
         <v>8.58</v>
       </c>
-    </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G144">
+        <f t="shared" si="2"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>2011</v>
       </c>
@@ -5705,6 +6283,10 @@
       </c>
       <c r="F145" s="62">
         <v>1.71</v>
+      </c>
+      <c r="G145">
+        <f t="shared" si="2"/>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>